<commit_message>
LSO List A: verified MFM points, drop Lancer's Sigil, lock 1,995/2000
- Pulled Knights points from BSData (= current MFM): Castellan 400, Crusader
  395, Cerastus Lancer 415, Armiger Helverin 140, Navigator 75; enhancements
  Blessed Plate 30, Judicant's Helm 25, Sanctuary 20. Resolves the 400-vs-425 hedge.
- Drop Bearer of the Lancer's Sigil (user: not worth it). Blessed Plate is the
  taken enhancement; Judicant's Helm + Sanctuary benched.
- Lock List A = 2 Castellan / 1 Lancer / 1 Crusader / 2 Armiger / Navigator +
  Blessed Plate = 1,995/2000 (2nd Armiger is the points-efficient fill vs
  wasting ~95 on one). Regenerated all three docs.

Still pending user confirmation: 'Rotate Ion Shields' NOT found anywhere in the
11E faction pack/core (flat 5++ vs ranged only) — the ~8 heist 'Rotate' mentions
+ the RULES entry are unchanged until confirmed.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reports & Plans/LSO-Knights-List-Decision.xlsx
+++ b/docs/Reports & Plans/LSO-Knights-List-Decision.xlsx
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="B7" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
@@ -1354,12 +1354,12 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>140 ea</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>Backfield 48" autocannons + cheap OC6 body / screen.</t>
+          <t>TWO backfield 48" autocannon platforms + OC6 screens — the points-efficient fill (a single Armiger wastes ~95 pts) + extra OC for the melee-heavy meta.</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>As written ~1825-1915 / 2000 with NO enhancements = the one concrete error. Add the 3 enhancements above to reach 2000 (Rotate is free). VERIFY exact points vs LIVE MFM before submitting — BSData prices Castellan 400, the app may be 425.</t>
+          <t>VERIFIED 1,995 / 2000: 2x Castellan 400 + Cerastus Lancer 415 + Crusader 395 + 2x Armiger Helverin 140 + Navigator 75 = 1,965, + Blessed Plate 30 = 1,995 (5 spare). Points from BSData = current MFM (Castellan 400 confirmed, not 425). NO Lancer's Sigil (rejected). The 2nd Armiger is the points-efficient fill — a single Armiger wastes ~95 pts the enhancement allowance can't absorb.</t>
         </is>
       </c>
     </row>
@@ -1405,51 +1405,51 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Bearer of the Lancer's Sigil</t>
+          <t>Blessed Plate  [TAKEN]</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cerastus Knight Lancer</t>
+          <t>a Knight Castellan</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>(25) Re-roll the Lancer's charge — with only ONE decapitation blade, guaranteeing its decisive charge is the highest-value 25 pts in the list.</t>
+          <t>(30) Castellan -&gt; T13: pushes S12-13 anti-tank (rail / ferrumite / lascannon / Caladius / thermal) from wounding on 4+ to 5+ — survivability for the key Volcano platform. The 2-Armiger build fits ~one enhancement; this is it.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>Blessed Plate</t>
+          <t>Bearer of the Judicant's Helm  [bench]</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Knight Castellan #1</t>
+          <t>a Knight Castellan</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>(30) Castellan -&gt; T13: the Volcano platform survives the incoming longer.</t>
+          <t>(25) [Ignores Cover] on a Castellan — stacks with Dominus +1-hit-in-terrain. Offensive alternative to Blessed Plate.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>Bearer of the Judicant's Helm</t>
+          <t>Sanctuary  [bench]</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Knight Castellan #2</t>
+          <t>a Knight Castellan</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>(25) [Ignores Cover] on a Castellan — stacks with Dominus +1-hit-in-terrain; beats intervening-terrain cover.</t>
+          <t>(20) 5++ invuln vs MELEE on one Castellan — patches the no-melee-invuln weakness (newly relevant: 11E has NO Rotate Ion Shields and Questoris have no melee save). Consider vs a melee-heavy field.</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>As written ~1825-1915 / 2000 with NO enhancements = the one concrete error. Add the 3 enhancements above to reach 2000 (Rotate is free). VERIFY exact points vs LIVE MFM before submitting — BSData prices Castellan 400, the app may be 425.</t>
+          <t>VERIFIED 1,995 / 2000: 2x Castellan 400 + Cerastus Lancer 415 + Crusader 395 + 2x Armiger Helverin 140 + Navigator 75 = 1,965, + Blessed Plate 30 = 1,995 (5 spare). Points from BSData = current MFM (Castellan 400 confirmed, not 425). NO Lancer's Sigil (rejected). The 2nd Armiger is the points-efficient fill — a single Armiger wastes ~95 pts the enhancement allowance can't absorb.</t>
         </is>
       </c>
     </row>
@@ -1665,51 +1665,51 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Bearer of the Lancer's Sigil</t>
+          <t>Blessed Plate  [TAKEN]</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cerastus Knight Lancer</t>
+          <t>a Knight Castellan</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>(25) Re-roll the Lancer's charge — with only ONE decapitation blade, guaranteeing its decisive charge is the highest-value 25 pts in the list.</t>
+          <t>(30) Castellan -&gt; T13: pushes S12-13 anti-tank (rail / ferrumite / lascannon / Caladius / thermal) from wounding on 4+ to 5+ — survivability for the key Volcano platform. The 2-Armiger build fits ~one enhancement; this is it.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>Blessed Plate</t>
+          <t>Bearer of the Judicant's Helm  [bench]</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Knight Castellan #1</t>
+          <t>a Knight Castellan</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>(30) Castellan -&gt; T13: the Volcano platform survives the incoming longer.</t>
+          <t>(25) [Ignores Cover] on a Castellan — stacks with Dominus +1-hit-in-terrain. Offensive alternative to Blessed Plate.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>Bearer of the Judicant's Helm</t>
+          <t>Sanctuary  [bench]</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Knight Castellan #2</t>
+          <t>a Knight Castellan</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>(25) [Ignores Cover] on a Castellan — stacks with Dominus +1-hit-in-terrain; beats intervening-terrain cover.</t>
+          <t>(20) 5++ invuln vs MELEE on one Castellan — patches the no-melee-invuln weakness (newly relevant: 11E has NO Rotate Ion Shields and Questoris have no melee save). Consider vs a melee-heavy field.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire the data-driven sim into the LSO decision docs (close the loop)
- mc_db_sim.results() exposes the sim for embedding.
- gen_lso_decision_xlsx.py: new "Sim Verification" sheet runs the sim live and
  tabulates A/B win% + enemy ak (ranged/melee) + my removal per archetype, so the
  decision workbook now carries BOTH the hand-analysis AND the simulation.
- Fix stale "Meta (n=75)" -> "n=70" sheet label.

Analysis -> DB -> sim -> decision doc is now one consistent, reproducible pipeline.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reports & Plans/LSO-Knights-List-Decision.xlsx
+++ b/docs/Reports & Plans/LSO-Knights-List-Decision.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DECISION" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta (n=75)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta (n=70)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List A" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List B" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matchups A vs B" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified Profiles" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sim Verification" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified Profiles" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2592,6 +2593,426 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>DATA-DRIVEN SIM — A vs B (my Knights' output computed from data/bsdata via wh.mathhammer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>800 games/(list x archetype). tools/mc_db_sim.py. akR/akM = enemy anti-Knight EV/turn (ranged/melee, DB where present else verified floor); rmv = my EV onto their priority target/turn. Confirms: A wins SHOOTING metas, B wins MELEE metas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Archetype</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>prev</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>akR</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>akM</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>A rmv</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>B rmv</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>A win%</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>B win%</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>Better list</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Emperor's Children (Defiler+swarm)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>41</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>31</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>47</v>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Orks (Green Tide horde)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>106</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>83</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>72</v>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>AdMech (Rad-Zone gunline)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>74</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>T'au (Retaliation alpha)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>37</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Necrons (Awakened C'tan)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>56</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Custodes (elite melee)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>34</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>34</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Blood Angels (jump alpha)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>89</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>65</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Dark Angels (Deathwing bricks)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>68</v>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Drukhari (Skysplinter)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Astra Militarum (superheavy)</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>43</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Fix remaining n=75 -> n=70 labels in decision Excel
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Reports & Plans/LSO-Knights-List-Decision.xlsx
+++ b/docs/Reports & Plans/LSO-Knights-List-Decision.xlsx
@@ -635,7 +635,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>PREVALENCE-WEIGHTED TALLY (n=75 top lists)</t>
+          <t>PREVALENCE-WEIGHTED TALLY (n=70 top lists)</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>WINNERS' META — top-finishing lists, ~14 late-July-2026 GTs (n=75)</t>
+          <t>WINNERS' META — top-finishing lists, ~14 late-July-2026 GTs (n=70)</t>
         </is>
       </c>
     </row>

</xml_diff>